<commit_message>
3 versao da lista brainstotming
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
@@ -1,42 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29930"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SI-2026\Projetos2SIPF\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D5180-3594-4B0C-954D-2A242D14B098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{1C2D5180-3594-4B0C-954D-2A242D14B098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C02F5DB-E209-4898-A6C7-5700E4BD043A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DO SISTEMA DE GERENCIAMENTO DE ESTACIONAMENTO</t>
-  </si>
-  <si>
-    <t>Id*</t>
-  </si>
-  <si>
-    <t>Nome do requisito</t>
-  </si>
-  <si>
-    <t>Descrição da regra de domínio (regra de negócio/de operação)</t>
   </si>
   <si>
     <r>
@@ -62,22 +64,70 @@
     </r>
   </si>
   <si>
+    <t>Id*</t>
+  </si>
+  <si>
+    <t>Nome do requisito</t>
+  </si>
+  <si>
+    <t>Descrição da regra de domínio (regra de negócio/de operação)</t>
+  </si>
+  <si>
+    <t>Rnf001</t>
+  </si>
+  <si>
     <t>Sistema deve rodar em interface WEB para PC/Note/Mobile</t>
   </si>
   <si>
-    <t>Rnf001</t>
-  </si>
-  <si>
     <t>Usar linguagem de programação para aplicações WEB</t>
   </si>
   <si>
+    <t>Rnf002</t>
+  </si>
+  <si>
+    <t>Padrão das telas do sistema</t>
+  </si>
+  <si>
+    <t>Fundo azul marinho com letras em branco, logo da empresa usuária do sistema no topo da tela do lado direito</t>
+  </si>
+  <si>
+    <t>Rnf003</t>
+  </si>
+  <si>
+    <t>Os dashboards gerenciais precisam ficar na mesma tela</t>
+  </si>
+  <si>
+    <t>Criar áreas separadas em janelas na tela de consulta</t>
+  </si>
+  <si>
+    <t>Rnf004</t>
+  </si>
+  <si>
+    <t>Disponibilidade Offline</t>
+  </si>
+  <si>
+    <t>O sistema deve operar localmente em caso de queda de link de internet</t>
+  </si>
+  <si>
+    <t>Rnf005</t>
+  </si>
+  <si>
+    <t>Conformidade LGPD</t>
+  </si>
+  <si>
+    <t>Criptografia de dados pessoais e opção de anonimização de histórico</t>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
     <t>Comunicar com sistemas de meio de pagamento</t>
   </si>
   <si>
     <t>Usar os protocolos de interface dos meios de pagamento CIELO, REDECARD e PIX</t>
   </si>
   <si>
-    <t>Rf001</t>
+    <t>Rf002</t>
   </si>
   <si>
     <t>Emissão de nota/cupom fiscal</t>
@@ -86,7 +136,7 @@
     <t>Integrar com impressora fiscal e sistema da Receita (Secretaria da Fazenda)</t>
   </si>
   <si>
-    <t>Rf002</t>
+    <t>Rf003</t>
   </si>
   <si>
     <t>Suporte para conveniados</t>
@@ -95,61 +145,43 @@
     <t>Tabela de preços específica para convênios com empresas</t>
   </si>
   <si>
-    <t>Rf003</t>
-  </si>
-  <si>
-    <t>Rnf002</t>
-  </si>
-  <si>
-    <t>Padrão das telas do sistema</t>
-  </si>
-  <si>
-    <t>Fundo azul marinho com letras em branco, logo da empresa usuária do sistema no topo da tela do lado direito</t>
+    <t>Rf004</t>
   </si>
   <si>
     <t>Dashboard de consulta de quantidade média de veículos por dia da semana</t>
   </si>
   <si>
+    <t>Mostrar um gráfico de barras com as datas no eixo X e quantidades no eixo Y</t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
     <t>Dashboard do dia de pico de cada mês no último ano</t>
   </si>
   <si>
+    <t>Mostrar um relatório em forma de tabela com os dias de pico de cada mês e a quantidade de carros movimentada no dia</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
     <t>Dashboard de valor faturado por dia/mês no último ano</t>
   </si>
   <si>
-    <t>Rnf003</t>
-  </si>
-  <si>
-    <t>Os dashboards gerenciais precisam ficar na mesma tela</t>
-  </si>
-  <si>
-    <t>Rf004</t>
-  </si>
-  <si>
-    <t>Rf005</t>
-  </si>
-  <si>
-    <t>Rf006</t>
-  </si>
-  <si>
-    <t>Criar áreas separadas em janelas na tela de consulta</t>
-  </si>
-  <si>
-    <t>Mostrar um gráfico de barras com as datas no eixo X e quantidades no eixo Y</t>
-  </si>
-  <si>
-    <t>Mostrar um relatório em forma de tabela com os dias de pico de cada mês e a quantidade de carros movimentada no dia</t>
-  </si>
-  <si>
     <t>Mostrar um gráfico de linhas com as datas no eixo X e os valores faturados no eixo Y</t>
   </si>
   <si>
+    <t>Rf007</t>
+  </si>
+  <si>
     <t>Notificação de proximidade do horário de fechamento</t>
   </si>
   <si>
     <t>Avisar por Whatsapp que o estacionamento vai fechar, com 1 mensagem aos 30 min antes, 1 aos 10 min antes</t>
   </si>
   <si>
-    <t>Rf007</t>
+    <t>Rf008</t>
   </si>
   <si>
     <t>Notificação do tempo de permanência</t>
@@ -158,7 +190,7 @@
     <t>A cada 30 min estacionado, enviar aviso por Whatsapp ao cliente com o tempo e o valor do momento</t>
   </si>
   <si>
-    <t>Rf008</t>
+    <t>Rf009</t>
   </si>
   <si>
     <t>Controle de status de ocupação de vagas</t>
@@ -167,7 +199,7 @@
     <t>Cada vaga tem status de ocupada ou livre</t>
   </si>
   <si>
-    <t>Rf009</t>
+    <t>Rf010</t>
   </si>
   <si>
     <t>Leitura automática de placas</t>
@@ -176,9 +208,6 @@
     <t>Vincular cadastro de veículo com placa, agilizando a entrada e saída</t>
   </si>
   <si>
-    <t>Rf010</t>
-  </si>
-  <si>
     <t>Rf011</t>
   </si>
   <si>
@@ -186,13 +215,91 @@
   </si>
   <si>
     <t>Permitir controlar mais de um estacionamento, suas vagas e movimentos</t>
+  </si>
+  <si>
+    <t>Rf012</t>
+  </si>
+  <si>
+    <t>Gestão de pagamento de Mensalistas</t>
+  </si>
+  <si>
+    <t>Controle de pagamentos com boleto, PIX ou Cartão e vencimentos</t>
+  </si>
+  <si>
+    <t>Rf013</t>
+  </si>
+  <si>
+    <t>Gestão de pagamento de avulsos</t>
+  </si>
+  <si>
+    <t>Controle de pagamentos com tabel de preços por dia/horário/permanência</t>
+  </si>
+  <si>
+    <t>Rd014</t>
+  </si>
+  <si>
+    <t>Gestão de Controle de Caixa</t>
+  </si>
+  <si>
+    <t>Exigir rotina de abertura e fechamento de caixa por cada usuario, registrando valor inicial e final do caixa.</t>
+  </si>
+  <si>
+    <t>Rf015</t>
+  </si>
+  <si>
+    <t>Medidas de segurança</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impedimento de fraudes por meio de registros com fotos e códigos </t>
+  </si>
+  <si>
+    <t>Rf016</t>
+  </si>
+  <si>
+    <t>Controle de vagas para carros eletricos</t>
+  </si>
+  <si>
+    <t>Mostrar quais vagas do estacionamento sao especificas para carros eletricos com carregador para poder usar</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Rf017</t>
+  </si>
+  <si>
+    <t>Bloqueio de mensalistas e conveniados por falta de pagamento</t>
+  </si>
+  <si>
+    <t>Após 15 das em atraso de mensalidade, bloquear a entrada (emitir aviso ao operador da recepção ou bloquear cancela)</t>
+  </si>
+  <si>
+    <t>e/</t>
+  </si>
+  <si>
+    <t>Rf018</t>
+  </si>
+  <si>
+    <t>Registro de Avarias</t>
+  </si>
+  <si>
+    <t>Registrar fotos do veículo na entrada para evitar falsas queixas de danos</t>
+  </si>
+  <si>
+    <t>Rf019</t>
+  </si>
+  <si>
+    <t>Vagas prioridade e compatibilidade</t>
+  </si>
+  <si>
+    <t>Apenas veículos com permissão podem ocupar vagas marcadas com EV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -563,193 +670,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="54.42578125" customWidth="1"/>
     <col min="3" max="3" width="126.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="1" t="s">
+    <row r="10" spans="1:3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:4">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>46</v>
       </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="17.25" customHeight="1">
+      <c r="A24" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D29" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -758,6 +1016,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007544514C3E525041A50FD90CCA057415" ma:contentTypeVersion="10" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="bf4730f3f1a762055629886e8f42d477">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b591360b-72bd-45d7-9362-d2d404a7b4f5" xmlns:ns3="e265a0ad-4171-4359-86dd-7b4a7d920c0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e150f1db5eef3c20961c9854c2263c4" ns2:_="" ns3:_="">
     <xsd:import namespace="b591360b-72bd-45d7-9362-d2d404a7b4f5"/>
@@ -946,15 +1213,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -967,11 +1225,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800DB960-F05E-4141-AFC3-FD43E9D5A7C9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D1F747B-A076-4329-9D35-44DBCC6CEFE3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D1F747B-A076-4329-9D35-44DBCC6CEFE3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800DB960-F05E-4141-AFC3-FD43E9D5A7C9}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>